<commit_message>
added admin email in excel
</commit_message>
<xml_diff>
--- a/Venues_Data.xlsx
+++ b/Venues_Data.xlsx
@@ -116,7 +116,7 @@
     <t>North</t>
   </si>
   <si>
-    <t>arnavp22.comp@coeptech.ac.in</t>
+    <t>dean.engineeringoffice@coeptech.ac.in</t>
   </si>
   <si>
     <t>NC 02</t>
@@ -580,7 +580,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -591,12 +591,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1003,7 +997,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="45">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1029,106 +1023,103 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="11" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="11" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="12" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="12" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="13" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="13" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="14" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="15" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="14" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="15" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="13" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="15" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="16" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="13" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="16" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="19" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="19" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="20" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="20" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="11" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="11" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="21" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="21" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="22" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="22" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="23" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="23" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -1139,9 +1130,6 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1448,27 +1436,27 @@
   <dimension ref="A1:U92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="43" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="44" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="44" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="44" width="27.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="44" width="38.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="44" width="41.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="45" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="45" width="15.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="45" width="14.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="43" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="44" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="44" width="58.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="46" width="31.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="46" width="66.7192857142857" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="46" width="30.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="46" width="29.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="44" width="29.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="46" width="30.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="46" width="35.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="46" width="29.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="44" width="29.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="42" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="43" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="43" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="43" width="27.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="43" width="38.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="43" width="41.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="44" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="44" width="15.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="44" width="14.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="42" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="43" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="43" width="58.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="43" width="31.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="43" width="66.7192857142857" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="43" width="30.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="43" width="29.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="43" width="29.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="43" width="30.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="43" width="35.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="43" width="29.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="43" width="29.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -1602,7 +1590,7 @@
       <c r="D3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F3" s="23" t="s">
@@ -1620,7 +1608,7 @@
       <c r="J3" s="22">
         <v>108</v>
       </c>
-      <c r="K3" s="25" t="s">
+      <c r="K3" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L3" s="21" t="s">
@@ -1655,7 +1643,7 @@
       <c r="D4" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F4" s="23" t="s">
@@ -1673,7 +1661,7 @@
       <c r="J4" s="22">
         <v>108</v>
       </c>
-      <c r="K4" s="25" t="s">
+      <c r="K4" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L4" s="21" t="s">
@@ -1708,7 +1696,7 @@
       <c r="D5" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F5" s="23" t="s">
@@ -1726,7 +1714,7 @@
       <c r="J5" s="22">
         <v>117</v>
       </c>
-      <c r="K5" s="25" t="s">
+      <c r="K5" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L5" s="21" t="s">
@@ -1761,7 +1749,7 @@
       <c r="D6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F6" s="23" t="s">
@@ -1779,27 +1767,27 @@
       <c r="J6" s="22">
         <v>111</v>
       </c>
-      <c r="K6" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L6" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M6" s="27" t="s">
+      <c r="K6" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L6" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="N6" s="28" t="s">
+      <c r="N6" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="O6" s="29" t="s">
+      <c r="O6" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="P6" s="28"/>
+      <c r="P6" s="27"/>
       <c r="Q6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R6" s="29"/>
-      <c r="S6" s="28"/>
+      <c r="R6" s="28"/>
+      <c r="S6" s="27"/>
       <c r="T6" s="11" t="s">
         <v>28</v>
       </c>
@@ -1820,7 +1808,7 @@
       <c r="D7" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F7" s="23" t="s">
@@ -1838,27 +1826,27 @@
       <c r="J7" s="22">
         <v>108</v>
       </c>
-      <c r="K7" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L7" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M7" s="27" t="s">
+      <c r="K7" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L7" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="N7" s="28" t="s">
+      <c r="N7" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="O7" s="29" t="s">
+      <c r="O7" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="P7" s="28"/>
+      <c r="P7" s="27"/>
       <c r="Q7" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R7" s="29"/>
-      <c r="S7" s="28"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="27"/>
       <c r="T7" s="11" t="s">
         <v>28</v>
       </c>
@@ -1879,7 +1867,7 @@
       <c r="D8" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F8" s="23" t="s">
@@ -1897,27 +1885,27 @@
       <c r="J8" s="22">
         <v>108</v>
       </c>
-      <c r="K8" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L8" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M8" s="30" t="s">
+      <c r="K8" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M8" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="N8" s="31" t="s">
+      <c r="N8" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="O8" s="32" t="s">
+      <c r="O8" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="P8" s="31"/>
+      <c r="P8" s="30"/>
       <c r="Q8" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R8" s="32"/>
-      <c r="S8" s="31"/>
+      <c r="R8" s="31"/>
+      <c r="S8" s="30"/>
       <c r="T8" s="11" t="s">
         <v>28</v>
       </c>
@@ -1938,7 +1926,7 @@
       <c r="D9" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F9" s="23" t="s">
@@ -1956,7 +1944,7 @@
       <c r="J9" s="22">
         <v>117</v>
       </c>
-      <c r="K9" s="25" t="s">
+      <c r="K9" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L9" s="21" t="s">
@@ -1991,7 +1979,7 @@
       <c r="D10" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="23" t="s">
@@ -2009,31 +1997,31 @@
       <c r="J10" s="22">
         <v>200</v>
       </c>
-      <c r="K10" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L10" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M10" s="33" t="s">
+      <c r="K10" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="N10" s="33" t="s">
+      <c r="N10" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="O10" s="30" t="s">
+      <c r="O10" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="P10" s="31" t="s">
+      <c r="P10" s="30" t="s">
         <v>47</v>
       </c>
       <c r="Q10" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R10" s="32" t="s">
+      <c r="R10" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="S10" s="31" t="s">
+      <c r="S10" s="30" t="s">
         <v>48</v>
       </c>
       <c r="T10" s="11" t="s">
@@ -2056,7 +2044,7 @@
       <c r="D11" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F11" s="23" t="s">
@@ -2074,7 +2062,7 @@
       <c r="J11" s="22">
         <v>200</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="K11" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L11" s="21" t="s">
@@ -2109,7 +2097,7 @@
       <c r="D12" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F12" s="23" t="s">
@@ -2127,7 +2115,7 @@
       <c r="J12" s="22">
         <v>108</v>
       </c>
-      <c r="K12" s="25" t="s">
+      <c r="K12" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L12" s="21" t="s">
@@ -2162,7 +2150,7 @@
       <c r="D13" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F13" s="23" t="s">
@@ -2180,7 +2168,7 @@
       <c r="J13" s="22">
         <v>108</v>
       </c>
-      <c r="K13" s="25" t="s">
+      <c r="K13" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L13" s="21" t="s">
@@ -2215,7 +2203,7 @@
       <c r="D14" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F14" s="23" t="s">
@@ -2233,7 +2221,7 @@
       <c r="J14" s="22">
         <v>108</v>
       </c>
-      <c r="K14" s="25" t="s">
+      <c r="K14" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L14" s="21" t="s">
@@ -2268,7 +2256,7 @@
       <c r="D15" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="24" t="s">
+      <c r="E15" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F15" s="23" t="s">
@@ -2286,21 +2274,21 @@
       <c r="J15" s="22">
         <v>117</v>
       </c>
-      <c r="K15" s="25" t="s">
+      <c r="K15" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L15" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M15" s="34"/>
-      <c r="N15" s="34"/>
-      <c r="O15" s="34"/>
-      <c r="P15" s="34"/>
+      <c r="M15" s="33"/>
+      <c r="N15" s="33"/>
+      <c r="O15" s="33"/>
+      <c r="P15" s="33"/>
       <c r="Q15" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R15" s="34"/>
-      <c r="S15" s="34"/>
+      <c r="R15" s="33"/>
+      <c r="S15" s="33"/>
       <c r="T15" s="11" t="s">
         <v>28</v>
       </c>
@@ -2321,7 +2309,7 @@
       <c r="D16" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="24" t="s">
+      <c r="E16" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F16" s="23" t="s">
@@ -2339,27 +2327,27 @@
       <c r="J16" s="22">
         <v>200</v>
       </c>
-      <c r="K16" s="25" t="s">
+      <c r="K16" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L16" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M16" s="29" t="s">
+      <c r="M16" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="N16" s="27" t="s">
+      <c r="N16" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="O16" s="27" t="s">
+      <c r="O16" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="P16" s="28"/>
+      <c r="P16" s="27"/>
       <c r="Q16" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R16" s="29"/>
-      <c r="S16" s="28"/>
+      <c r="R16" s="28"/>
+      <c r="S16" s="27"/>
       <c r="T16" s="11" t="s">
         <v>28</v>
       </c>
@@ -2380,7 +2368,7 @@
       <c r="D17" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="3" t="s">
         <v>60</v>
       </c>
       <c r="F17" s="23" t="s">
@@ -2398,27 +2386,27 @@
       <c r="J17" s="22">
         <v>50</v>
       </c>
-      <c r="K17" s="25" t="s">
+      <c r="K17" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L17" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M17" s="29" t="s">
+      <c r="M17" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="N17" s="27" t="s">
+      <c r="N17" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="O17" s="27" t="s">
+      <c r="O17" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="P17" s="28"/>
+      <c r="P17" s="27"/>
       <c r="Q17" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R17" s="29"/>
-      <c r="S17" s="28"/>
+      <c r="R17" s="28"/>
+      <c r="S17" s="27"/>
       <c r="T17" s="11" t="s">
         <v>28</v>
       </c>
@@ -2439,7 +2427,7 @@
       <c r="D18" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="3" t="s">
         <v>60</v>
       </c>
       <c r="F18" s="23" t="s">
@@ -2457,27 +2445,27 @@
       <c r="J18" s="22">
         <v>30</v>
       </c>
-      <c r="K18" s="25" t="s">
+      <c r="K18" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L18" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M18" s="32" t="s">
+      <c r="M18" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="N18" s="30" t="s">
+      <c r="N18" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="O18" s="30" t="s">
+      <c r="O18" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="P18" s="31"/>
+      <c r="P18" s="30"/>
       <c r="Q18" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R18" s="32"/>
-      <c r="S18" s="31"/>
+      <c r="R18" s="31"/>
+      <c r="S18" s="30"/>
       <c r="T18" s="11" t="s">
         <v>28</v>
       </c>
@@ -2498,7 +2486,7 @@
       <c r="D19" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="3" t="s">
         <v>60</v>
       </c>
       <c r="F19" s="23" t="s">
@@ -2516,21 +2504,21 @@
       <c r="J19" s="22">
         <v>50</v>
       </c>
-      <c r="K19" s="25" t="s">
+      <c r="K19" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L19" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M19" s="35"/>
-      <c r="N19" s="35"/>
-      <c r="O19" s="35"/>
-      <c r="P19" s="35"/>
+      <c r="M19" s="34"/>
+      <c r="N19" s="34"/>
+      <c r="O19" s="34"/>
+      <c r="P19" s="34"/>
       <c r="Q19" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R19" s="35"/>
-      <c r="S19" s="35"/>
+      <c r="R19" s="34"/>
+      <c r="S19" s="34"/>
       <c r="T19" s="11" t="s">
         <v>28</v>
       </c>
@@ -2551,7 +2539,7 @@
       <c r="D20" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="3" t="s">
         <v>65</v>
       </c>
       <c r="F20" s="23" t="s">
@@ -2569,7 +2557,7 @@
       <c r="J20" s="22">
         <v>30</v>
       </c>
-      <c r="K20" s="25" t="s">
+      <c r="K20" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L20" s="21" t="s">
@@ -2604,7 +2592,7 @@
       <c r="D21" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="24" t="s">
+      <c r="E21" s="3" t="s">
         <v>65</v>
       </c>
       <c r="F21" s="23" t="s">
@@ -2622,7 +2610,7 @@
       <c r="J21" s="22">
         <v>30</v>
       </c>
-      <c r="K21" s="25" t="s">
+      <c r="K21" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L21" s="21" t="s">
@@ -2657,7 +2645,7 @@
       <c r="D22" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="3" t="s">
         <v>65</v>
       </c>
       <c r="F22" s="23" t="s">
@@ -2675,7 +2663,7 @@
       <c r="J22" s="22">
         <v>30</v>
       </c>
-      <c r="K22" s="25" t="s">
+      <c r="K22" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="21" t="s">
@@ -2710,7 +2698,7 @@
       <c r="D23" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="3" t="s">
         <v>65</v>
       </c>
       <c r="F23" s="23" t="s">
@@ -2728,7 +2716,7 @@
       <c r="J23" s="22">
         <v>30</v>
       </c>
-      <c r="K23" s="25" t="s">
+      <c r="K23" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L23" s="21" t="s">
@@ -2763,7 +2751,7 @@
       <c r="D24" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="3" t="s">
         <v>65</v>
       </c>
       <c r="F24" s="23" t="s">
@@ -2781,7 +2769,7 @@
       <c r="J24" s="22">
         <v>56</v>
       </c>
-      <c r="K24" s="25" t="s">
+      <c r="K24" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L24" s="21" t="s">
@@ -2816,7 +2804,7 @@
       <c r="D25" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="24" t="s">
+      <c r="E25" s="3" t="s">
         <v>65</v>
       </c>
       <c r="F25" s="23" t="s">
@@ -2834,7 +2822,7 @@
       <c r="J25" s="22">
         <v>30</v>
       </c>
-      <c r="K25" s="25" t="s">
+      <c r="K25" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L25" s="21" t="s">
@@ -2869,7 +2857,7 @@
       <c r="D26" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="3" t="s">
         <v>65</v>
       </c>
       <c r="F26" s="23" t="s">
@@ -2887,7 +2875,7 @@
       <c r="J26" s="22">
         <v>100</v>
       </c>
-      <c r="K26" s="25" t="s">
+      <c r="K26" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L26" s="21" t="s">
@@ -2922,7 +2910,7 @@
       <c r="D27" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="24" t="s">
+      <c r="E27" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F27" s="23" t="s">
@@ -2940,7 +2928,7 @@
       <c r="J27" s="22">
         <v>100</v>
       </c>
-      <c r="K27" s="25" t="s">
+      <c r="K27" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L27" s="21" t="s">
@@ -2975,7 +2963,7 @@
       <c r="D28" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E28" s="24" t="s">
+      <c r="E28" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F28" s="23" t="s">
@@ -2993,7 +2981,7 @@
       <c r="J28" s="22">
         <v>120</v>
       </c>
-      <c r="K28" s="25" t="s">
+      <c r="K28" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L28" s="21" t="s">
@@ -3028,7 +3016,7 @@
       <c r="D29" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E29" s="24" t="s">
+      <c r="E29" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F29" s="23" t="s">
@@ -3046,7 +3034,7 @@
       <c r="J29" s="22">
         <v>135</v>
       </c>
-      <c r="K29" s="25" t="s">
+      <c r="K29" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L29" s="21" t="s">
@@ -3081,7 +3069,7 @@
       <c r="D30" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E30" s="24" t="s">
+      <c r="E30" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F30" s="23" t="s">
@@ -3099,7 +3087,7 @@
       <c r="J30" s="22">
         <v>50</v>
       </c>
-      <c r="K30" s="25" t="s">
+      <c r="K30" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L30" s="21" t="s">
@@ -3134,7 +3122,7 @@
       <c r="D31" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E31" s="24" t="s">
+      <c r="E31" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F31" s="23" t="s">
@@ -3152,7 +3140,7 @@
       <c r="J31" s="22">
         <v>100</v>
       </c>
-      <c r="K31" s="25" t="s">
+      <c r="K31" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L31" s="21" t="s">
@@ -3187,7 +3175,7 @@
       <c r="D32" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E32" s="24" t="s">
+      <c r="E32" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F32" s="23" t="s">
@@ -3205,7 +3193,7 @@
       <c r="J32" s="22">
         <v>50</v>
       </c>
-      <c r="K32" s="25" t="s">
+      <c r="K32" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L32" s="21" t="s">
@@ -3240,7 +3228,7 @@
       <c r="D33" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E33" s="24" t="s">
+      <c r="E33" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F33" s="23" t="s">
@@ -3258,7 +3246,7 @@
       <c r="J33" s="22">
         <v>70</v>
       </c>
-      <c r="K33" s="25" t="s">
+      <c r="K33" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L33" s="21" t="s">
@@ -3293,7 +3281,7 @@
       <c r="D34" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E34" s="24" t="s">
+      <c r="E34" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F34" s="23" t="s">
@@ -3311,7 +3299,7 @@
       <c r="J34" s="22">
         <v>30</v>
       </c>
-      <c r="K34" s="25" t="s">
+      <c r="K34" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L34" s="21" t="s">
@@ -3346,7 +3334,7 @@
       <c r="D35" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E35" s="24" t="s">
+      <c r="E35" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F35" s="23" t="s">
@@ -3364,21 +3352,21 @@
       <c r="J35" s="22">
         <v>20</v>
       </c>
-      <c r="K35" s="25" t="s">
+      <c r="K35" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L35" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M35" s="35"/>
-      <c r="N35" s="35"/>
-      <c r="O35" s="35"/>
-      <c r="P35" s="35"/>
+      <c r="M35" s="34"/>
+      <c r="N35" s="34"/>
+      <c r="O35" s="34"/>
+      <c r="P35" s="34"/>
       <c r="Q35" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R35" s="35"/>
-      <c r="S35" s="35"/>
+      <c r="R35" s="34"/>
+      <c r="S35" s="34"/>
       <c r="T35" s="11" t="s">
         <v>28</v>
       </c>
@@ -3399,7 +3387,7 @@
       <c r="D36" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E36" s="24" t="s">
+      <c r="E36" s="3" t="s">
         <v>75</v>
       </c>
       <c r="F36" s="23" t="s">
@@ -3417,7 +3405,7 @@
       <c r="J36" s="22">
         <v>175</v>
       </c>
-      <c r="K36" s="25" t="s">
+      <c r="K36" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L36" s="21" t="s">
@@ -3452,7 +3440,7 @@
       <c r="D37" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E37" s="24" t="s">
+      <c r="E37" s="3" t="s">
         <v>87</v>
       </c>
       <c r="F37" s="23" t="s">
@@ -3470,7 +3458,7 @@
       <c r="J37" s="22">
         <v>80</v>
       </c>
-      <c r="K37" s="25" t="s">
+      <c r="K37" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L37" s="21" t="s">
@@ -3505,7 +3493,7 @@
       <c r="D38" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E38" s="24" t="s">
+      <c r="E38" s="3" t="s">
         <v>87</v>
       </c>
       <c r="F38" s="23" t="s">
@@ -3523,7 +3511,7 @@
       <c r="J38" s="22">
         <v>84</v>
       </c>
-      <c r="K38" s="25" t="s">
+      <c r="K38" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L38" s="21" t="s">
@@ -3558,7 +3546,7 @@
       <c r="D39" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E39" s="24" t="s">
+      <c r="E39" s="3" t="s">
         <v>87</v>
       </c>
       <c r="F39" s="23" t="s">
@@ -3576,7 +3564,7 @@
       <c r="J39" s="22">
         <v>60</v>
       </c>
-      <c r="K39" s="25" t="s">
+      <c r="K39" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L39" s="21" t="s">
@@ -3611,7 +3599,7 @@
       <c r="D40" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E40" s="24" t="s">
+      <c r="E40" s="3" t="s">
         <v>87</v>
       </c>
       <c r="F40" s="23" t="s">
@@ -3629,7 +3617,7 @@
       <c r="J40" s="22">
         <v>80</v>
       </c>
-      <c r="K40" s="25" t="s">
+      <c r="K40" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L40" s="21" t="s">
@@ -3664,7 +3652,7 @@
       <c r="D41" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E41" s="24" t="s">
+      <c r="E41" s="3" t="s">
         <v>87</v>
       </c>
       <c r="F41" s="23" t="s">
@@ -3682,21 +3670,21 @@
       <c r="J41" s="22">
         <v>60</v>
       </c>
-      <c r="K41" s="25" t="s">
+      <c r="K41" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L41" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M41" s="35"/>
-      <c r="N41" s="35"/>
-      <c r="O41" s="35"/>
-      <c r="P41" s="35"/>
+      <c r="M41" s="34"/>
+      <c r="N41" s="34"/>
+      <c r="O41" s="34"/>
+      <c r="P41" s="34"/>
       <c r="Q41" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R41" s="35"/>
-      <c r="S41" s="35"/>
+      <c r="R41" s="34"/>
+      <c r="S41" s="34"/>
       <c r="T41" s="11" t="s">
         <v>28</v>
       </c>
@@ -3717,7 +3705,7 @@
       <c r="D42" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E42" s="24" t="s">
+      <c r="E42" s="3" t="s">
         <v>87</v>
       </c>
       <c r="F42" s="23" t="s">
@@ -3735,7 +3723,7 @@
       <c r="J42" s="22">
         <v>40</v>
       </c>
-      <c r="K42" s="25" t="s">
+      <c r="K42" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L42" s="21" t="s">
@@ -3770,7 +3758,7 @@
       <c r="D43" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E43" s="24" t="s">
+      <c r="E43" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F43" s="23" t="s">
@@ -3782,7 +3770,7 @@
       <c r="J43" s="22">
         <v>80</v>
       </c>
-      <c r="K43" s="25" t="s">
+      <c r="K43" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L43" s="21" t="s">
@@ -3823,7 +3811,7 @@
       <c r="D44" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E44" s="24" t="s">
+      <c r="E44" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F44" s="23" t="s">
@@ -3835,7 +3823,7 @@
       <c r="J44" s="22">
         <v>80</v>
       </c>
-      <c r="K44" s="25" t="s">
+      <c r="K44" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L44" s="21" t="s">
@@ -3876,7 +3864,7 @@
       <c r="D45" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E45" s="24" t="s">
+      <c r="E45" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F45" s="23" t="s">
@@ -3888,7 +3876,7 @@
       <c r="J45" s="22">
         <v>80</v>
       </c>
-      <c r="K45" s="25" t="s">
+      <c r="K45" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L45" s="21" t="s">
@@ -3927,7 +3915,7 @@
       <c r="D46" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E46" s="24" t="s">
+      <c r="E46" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F46" s="23" t="s">
@@ -3939,7 +3927,7 @@
       <c r="J46" s="22">
         <v>80</v>
       </c>
-      <c r="K46" s="25" t="s">
+      <c r="K46" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L46" s="21" t="s">
@@ -3974,7 +3962,7 @@
       <c r="D47" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E47" s="24" t="s">
+      <c r="E47" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F47" s="23" t="s">
@@ -3986,27 +3974,27 @@
       <c r="J47" s="22">
         <v>80</v>
       </c>
-      <c r="K47" s="25" t="s">
+      <c r="K47" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L47" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M47" s="35" t="s">
+      <c r="M47" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="N47" s="35" t="s">
+      <c r="N47" s="34" t="s">
         <v>108</v>
       </c>
-      <c r="O47" s="35" t="s">
+      <c r="O47" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="P47" s="35"/>
+      <c r="P47" s="34"/>
       <c r="Q47" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R47" s="35"/>
-      <c r="S47" s="35"/>
+      <c r="R47" s="34"/>
+      <c r="S47" s="34"/>
       <c r="T47" s="11" t="s">
         <v>28</v>
       </c>
@@ -4027,7 +4015,7 @@
       <c r="D48" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E48" s="24" t="s">
+      <c r="E48" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F48" s="23" t="s">
@@ -4039,7 +4027,7 @@
       <c r="J48" s="22">
         <v>20</v>
       </c>
-      <c r="K48" s="25" t="s">
+      <c r="K48" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L48" s="21" t="s">
@@ -4074,7 +4062,7 @@
       <c r="D49" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E49" s="24" t="s">
+      <c r="E49" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F49" s="23" t="s">
@@ -4086,7 +4074,7 @@
       <c r="J49" s="22">
         <v>80</v>
       </c>
-      <c r="K49" s="25" t="s">
+      <c r="K49" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L49" s="21" t="s">
@@ -4121,7 +4109,7 @@
       <c r="D50" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E50" s="24" t="s">
+      <c r="E50" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F50" s="23" t="s">
@@ -4133,7 +4121,7 @@
       <c r="J50" s="22">
         <v>80</v>
       </c>
-      <c r="K50" s="25" t="s">
+      <c r="K50" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L50" s="21" t="s">
@@ -4168,7 +4156,7 @@
       <c r="D51" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E51" s="24" t="s">
+      <c r="E51" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F51" s="23" t="s">
@@ -4180,7 +4168,7 @@
       <c r="J51" s="22">
         <v>80</v>
       </c>
-      <c r="K51" s="25" t="s">
+      <c r="K51" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L51" s="21" t="s">
@@ -4215,7 +4203,7 @@
       <c r="D52" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E52" s="24" t="s">
+      <c r="E52" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F52" s="23" t="s">
@@ -4227,21 +4215,21 @@
       <c r="J52" s="22">
         <v>24</v>
       </c>
-      <c r="K52" s="25" t="s">
+      <c r="K52" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L52" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M52" s="35"/>
-      <c r="N52" s="35"/>
-      <c r="O52" s="35"/>
-      <c r="P52" s="35"/>
+      <c r="M52" s="34"/>
+      <c r="N52" s="34"/>
+      <c r="O52" s="34"/>
+      <c r="P52" s="34"/>
       <c r="Q52" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R52" s="35"/>
-      <c r="S52" s="35"/>
+      <c r="R52" s="34"/>
+      <c r="S52" s="34"/>
       <c r="T52" s="11" t="s">
         <v>28</v>
       </c>
@@ -4262,7 +4250,7 @@
       <c r="D53" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E53" s="24" t="s">
+      <c r="E53" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F53" s="23" t="s">
@@ -4274,7 +4262,7 @@
       <c r="J53" s="22">
         <v>24</v>
       </c>
-      <c r="K53" s="25" t="s">
+      <c r="K53" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L53" s="21" t="s">
@@ -4309,7 +4297,7 @@
       <c r="D54" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E54" s="24" t="s">
+      <c r="E54" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F54" s="23" t="s">
@@ -4321,7 +4309,7 @@
       <c r="J54" s="22">
         <v>150</v>
       </c>
-      <c r="K54" s="25" t="s">
+      <c r="K54" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L54" s="21" t="s">
@@ -4356,7 +4344,7 @@
       <c r="D55" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E55" s="24" t="s">
+      <c r="E55" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F55" s="23" t="s">
@@ -4368,7 +4356,7 @@
       <c r="J55" s="22">
         <v>150</v>
       </c>
-      <c r="K55" s="25" t="s">
+      <c r="K55" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L55" s="21" t="s">
@@ -4403,7 +4391,7 @@
       <c r="D56" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E56" s="24" t="s">
+      <c r="E56" s="3" t="s">
         <v>120</v>
       </c>
       <c r="F56" s="23" t="s">
@@ -4421,7 +4409,7 @@
       <c r="J56" s="22">
         <v>135</v>
       </c>
-      <c r="K56" s="25" t="s">
+      <c r="K56" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L56" s="21" t="s">
@@ -4456,7 +4444,7 @@
       <c r="D57" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E57" s="24" t="s">
+      <c r="E57" s="3" t="s">
         <v>120</v>
       </c>
       <c r="F57" s="23" t="s">
@@ -4474,7 +4462,7 @@
       <c r="J57" s="22">
         <v>35</v>
       </c>
-      <c r="K57" s="25" t="s">
+      <c r="K57" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L57" s="21" t="s">
@@ -4509,7 +4497,7 @@
       <c r="D58" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E58" s="24" t="s">
+      <c r="E58" s="3" t="s">
         <v>120</v>
       </c>
       <c r="F58" s="23" t="s">
@@ -4527,7 +4515,7 @@
       <c r="J58" s="22">
         <v>60</v>
       </c>
-      <c r="K58" s="25" t="s">
+      <c r="K58" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L58" s="21" t="s">
@@ -4562,7 +4550,7 @@
       <c r="D59" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E59" s="24" t="s">
+      <c r="E59" s="3" t="s">
         <v>120</v>
       </c>
       <c r="F59" s="23" t="s">
@@ -4580,7 +4568,7 @@
       <c r="J59" s="22">
         <v>40</v>
       </c>
-      <c r="K59" s="25" t="s">
+      <c r="K59" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L59" s="21" t="s">
@@ -4615,7 +4603,7 @@
       <c r="D60" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E60" s="24" t="s">
+      <c r="E60" s="3" t="s">
         <v>120</v>
       </c>
       <c r="F60" s="23" t="s">
@@ -4633,7 +4621,7 @@
       <c r="J60" s="22">
         <v>100</v>
       </c>
-      <c r="K60" s="25" t="s">
+      <c r="K60" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L60" s="21" t="s">
@@ -4668,7 +4656,7 @@
       <c r="D61" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E61" s="24" t="s">
+      <c r="E61" s="3" t="s">
         <v>120</v>
       </c>
       <c r="F61" s="23" t="s">
@@ -4686,7 +4674,7 @@
       <c r="J61" s="22">
         <v>50</v>
       </c>
-      <c r="K61" s="25" t="s">
+      <c r="K61" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L61" s="21" t="s">
@@ -4721,7 +4709,7 @@
       <c r="D62" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E62" s="24" t="s">
+      <c r="E62" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F62" s="23" t="s">
@@ -4739,7 +4727,7 @@
       <c r="J62" s="22">
         <v>95</v>
       </c>
-      <c r="K62" s="25" t="s">
+      <c r="K62" s="24" t="s">
         <v>25</v>
       </c>
       <c r="L62" s="21" t="s">
@@ -4774,7 +4762,7 @@
       <c r="D63" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E63" s="24" t="s">
+      <c r="E63" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F63" s="23" t="s">
@@ -4792,22 +4780,22 @@
       <c r="J63" s="22">
         <v>70</v>
       </c>
-      <c r="K63" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L63" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M63" s="36"/>
-      <c r="N63" s="37"/>
-      <c r="O63" s="37"/>
-      <c r="P63" s="38"/>
+      <c r="K63" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L63" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M63" s="35"/>
+      <c r="N63" s="36"/>
+      <c r="O63" s="36"/>
+      <c r="P63" s="37"/>
       <c r="Q63" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R63" s="39"/>
-      <c r="S63" s="37"/>
-      <c r="T63" s="38"/>
+      <c r="R63" s="38"/>
+      <c r="S63" s="36"/>
+      <c r="T63" s="37"/>
       <c r="U63" s="11" t="s">
         <v>29</v>
       </c>
@@ -4825,7 +4813,7 @@
       <c r="D64" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E64" s="24" t="s">
+      <c r="E64" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F64" s="23" t="s">
@@ -4843,22 +4831,22 @@
       <c r="J64" s="22">
         <v>70</v>
       </c>
-      <c r="K64" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L64" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M64" s="40"/>
+      <c r="K64" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L64" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M64" s="39"/>
       <c r="N64" s="23"/>
       <c r="O64" s="23"/>
-      <c r="P64" s="41"/>
+      <c r="P64" s="40"/>
       <c r="Q64" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R64" s="42"/>
+      <c r="R64" s="41"/>
       <c r="S64" s="23"/>
-      <c r="T64" s="41"/>
+      <c r="T64" s="40"/>
       <c r="U64" s="11" t="s">
         <v>29</v>
       </c>
@@ -4876,7 +4864,7 @@
       <c r="D65" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E65" s="24" t="s">
+      <c r="E65" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F65" s="23" t="s">
@@ -4894,22 +4882,22 @@
       <c r="J65" s="22">
         <v>20</v>
       </c>
-      <c r="K65" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L65" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M65" s="40"/>
+      <c r="K65" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L65" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M65" s="39"/>
       <c r="N65" s="23"/>
       <c r="O65" s="23"/>
-      <c r="P65" s="41"/>
+      <c r="P65" s="40"/>
       <c r="Q65" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R65" s="42"/>
+      <c r="R65" s="41"/>
       <c r="S65" s="23"/>
-      <c r="T65" s="41"/>
+      <c r="T65" s="40"/>
       <c r="U65" s="11" t="s">
         <v>29</v>
       </c>
@@ -4927,7 +4915,7 @@
       <c r="D66" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E66" s="24" t="s">
+      <c r="E66" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F66" s="23" t="s">
@@ -4945,22 +4933,22 @@
       <c r="J66" s="22">
         <v>20</v>
       </c>
-      <c r="K66" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L66" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M66" s="40"/>
+      <c r="K66" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L66" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M66" s="39"/>
       <c r="N66" s="23"/>
       <c r="O66" s="23"/>
-      <c r="P66" s="41"/>
+      <c r="P66" s="40"/>
       <c r="Q66" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R66" s="42"/>
+      <c r="R66" s="41"/>
       <c r="S66" s="23"/>
-      <c r="T66" s="41"/>
+      <c r="T66" s="40"/>
       <c r="U66" s="11" t="s">
         <v>29</v>
       </c>
@@ -4978,7 +4966,7 @@
       <c r="D67" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E67" s="24" t="s">
+      <c r="E67" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F67" s="23" t="s">
@@ -4996,22 +4984,22 @@
       <c r="J67" s="22">
         <v>25</v>
       </c>
-      <c r="K67" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L67" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M67" s="40"/>
+      <c r="K67" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L67" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M67" s="39"/>
       <c r="N67" s="23"/>
       <c r="O67" s="23"/>
-      <c r="P67" s="41"/>
+      <c r="P67" s="40"/>
       <c r="Q67" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R67" s="42"/>
+      <c r="R67" s="41"/>
       <c r="S67" s="23"/>
-      <c r="T67" s="41"/>
+      <c r="T67" s="40"/>
       <c r="U67" s="11" t="s">
         <v>29</v>
       </c>
@@ -5029,7 +5017,7 @@
       <c r="D68" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E68" s="24" t="s">
+      <c r="E68" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F68" s="23" t="s">
@@ -5047,22 +5035,22 @@
       <c r="J68" s="22">
         <v>64</v>
       </c>
-      <c r="K68" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L68" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M68" s="40"/>
+      <c r="K68" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L68" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M68" s="39"/>
       <c r="N68" s="23"/>
       <c r="O68" s="23"/>
-      <c r="P68" s="41"/>
+      <c r="P68" s="40"/>
       <c r="Q68" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R68" s="42"/>
+      <c r="R68" s="41"/>
       <c r="S68" s="23"/>
-      <c r="T68" s="41"/>
+      <c r="T68" s="40"/>
       <c r="U68" s="11" t="s">
         <v>29</v>
       </c>
@@ -5080,7 +5068,7 @@
       <c r="D69" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E69" s="24" t="s">
+      <c r="E69" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F69" s="23" t="s">
@@ -5098,22 +5086,22 @@
       <c r="J69" s="22">
         <v>45</v>
       </c>
-      <c r="K69" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L69" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M69" s="40"/>
+      <c r="K69" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L69" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M69" s="39"/>
       <c r="N69" s="23"/>
       <c r="O69" s="23"/>
-      <c r="P69" s="41"/>
+      <c r="P69" s="40"/>
       <c r="Q69" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R69" s="42"/>
+      <c r="R69" s="41"/>
       <c r="S69" s="23"/>
-      <c r="T69" s="41"/>
+      <c r="T69" s="40"/>
       <c r="U69" s="11" t="s">
         <v>29</v>
       </c>
@@ -5131,7 +5119,7 @@
       <c r="D70" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E70" s="24" t="s">
+      <c r="E70" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F70" s="23" t="s">
@@ -5149,22 +5137,22 @@
       <c r="J70" s="22">
         <v>25</v>
       </c>
-      <c r="K70" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L70" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M70" s="40"/>
+      <c r="K70" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L70" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M70" s="39"/>
       <c r="N70" s="23"/>
       <c r="O70" s="23"/>
-      <c r="P70" s="41"/>
+      <c r="P70" s="40"/>
       <c r="Q70" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R70" s="42"/>
+      <c r="R70" s="41"/>
       <c r="S70" s="23"/>
-      <c r="T70" s="41"/>
+      <c r="T70" s="40"/>
       <c r="U70" s="11" t="s">
         <v>29</v>
       </c>
@@ -5182,7 +5170,7 @@
       <c r="D71" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E71" s="24" t="s">
+      <c r="E71" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F71" s="23" t="s">
@@ -5200,22 +5188,22 @@
       <c r="J71" s="22">
         <v>90</v>
       </c>
-      <c r="K71" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L71" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M71" s="40"/>
+      <c r="K71" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L71" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M71" s="39"/>
       <c r="N71" s="23"/>
       <c r="O71" s="23"/>
-      <c r="P71" s="41"/>
+      <c r="P71" s="40"/>
       <c r="Q71" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R71" s="42"/>
+      <c r="R71" s="41"/>
       <c r="S71" s="23"/>
-      <c r="T71" s="41"/>
+      <c r="T71" s="40"/>
       <c r="U71" s="11" t="s">
         <v>29</v>
       </c>
@@ -5233,7 +5221,7 @@
       <c r="D72" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E72" s="24" t="s">
+      <c r="E72" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F72" s="23" t="s">
@@ -5251,22 +5239,22 @@
       <c r="J72" s="22">
         <v>20</v>
       </c>
-      <c r="K72" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L72" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M72" s="40"/>
+      <c r="K72" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L72" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M72" s="39"/>
       <c r="N72" s="23"/>
       <c r="O72" s="23"/>
-      <c r="P72" s="41"/>
+      <c r="P72" s="40"/>
       <c r="Q72" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R72" s="42"/>
+      <c r="R72" s="41"/>
       <c r="S72" s="23"/>
-      <c r="T72" s="41"/>
+      <c r="T72" s="40"/>
       <c r="U72" s="11" t="s">
         <v>29</v>
       </c>
@@ -5284,7 +5272,7 @@
       <c r="D73" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E73" s="24" t="s">
+      <c r="E73" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F73" s="23" t="s">
@@ -5302,22 +5290,22 @@
       <c r="J73" s="22">
         <v>25</v>
       </c>
-      <c r="K73" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L73" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M73" s="40"/>
+      <c r="K73" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L73" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M73" s="39"/>
       <c r="N73" s="23"/>
       <c r="O73" s="23"/>
-      <c r="P73" s="41"/>
+      <c r="P73" s="40"/>
       <c r="Q73" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R73" s="42"/>
+      <c r="R73" s="41"/>
       <c r="S73" s="23"/>
-      <c r="T73" s="41"/>
+      <c r="T73" s="40"/>
       <c r="U73" s="11" t="s">
         <v>29</v>
       </c>
@@ -5335,7 +5323,7 @@
       <c r="D74" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E74" s="24" t="s">
+      <c r="E74" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F74" s="23" t="s">
@@ -5353,22 +5341,22 @@
       <c r="J74" s="22">
         <v>35</v>
       </c>
-      <c r="K74" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L74" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M74" s="40"/>
+      <c r="K74" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L74" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M74" s="39"/>
       <c r="N74" s="23"/>
       <c r="O74" s="23"/>
-      <c r="P74" s="41"/>
+      <c r="P74" s="40"/>
       <c r="Q74" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R74" s="42"/>
+      <c r="R74" s="41"/>
       <c r="S74" s="23"/>
-      <c r="T74" s="41"/>
+      <c r="T74" s="40"/>
       <c r="U74" s="11" t="s">
         <v>29</v>
       </c>
@@ -5386,7 +5374,7 @@
       <c r="D75" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E75" s="24" t="s">
+      <c r="E75" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F75" s="23" t="s">
@@ -5404,22 +5392,22 @@
       <c r="J75" s="22">
         <v>100</v>
       </c>
-      <c r="K75" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L75" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M75" s="40"/>
+      <c r="K75" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L75" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M75" s="39"/>
       <c r="N75" s="23"/>
       <c r="O75" s="23"/>
-      <c r="P75" s="41"/>
+      <c r="P75" s="40"/>
       <c r="Q75" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R75" s="42"/>
+      <c r="R75" s="41"/>
       <c r="S75" s="23"/>
-      <c r="T75" s="41"/>
+      <c r="T75" s="40"/>
       <c r="U75" s="11" t="s">
         <v>29</v>
       </c>
@@ -5437,7 +5425,7 @@
       <c r="D76" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E76" s="24" t="s">
+      <c r="E76" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F76" s="23" t="s">
@@ -5455,22 +5443,22 @@
       <c r="J76" s="22">
         <v>20</v>
       </c>
-      <c r="K76" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L76" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M76" s="40"/>
+      <c r="K76" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L76" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M76" s="39"/>
       <c r="N76" s="23"/>
       <c r="O76" s="23"/>
-      <c r="P76" s="41"/>
+      <c r="P76" s="40"/>
       <c r="Q76" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R76" s="42"/>
+      <c r="R76" s="41"/>
       <c r="S76" s="23"/>
-      <c r="T76" s="41"/>
+      <c r="T76" s="40"/>
       <c r="U76" s="11" t="s">
         <v>29</v>
       </c>
@@ -5488,7 +5476,7 @@
       <c r="D77" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E77" s="24" t="s">
+      <c r="E77" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F77" s="23" t="s">
@@ -5506,22 +5494,22 @@
       <c r="J77" s="22">
         <v>95</v>
       </c>
-      <c r="K77" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L77" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M77" s="40"/>
+      <c r="K77" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L77" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M77" s="39"/>
       <c r="N77" s="23"/>
       <c r="O77" s="23"/>
-      <c r="P77" s="41"/>
+      <c r="P77" s="40"/>
       <c r="Q77" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R77" s="42"/>
+      <c r="R77" s="41"/>
       <c r="S77" s="23"/>
-      <c r="T77" s="41"/>
+      <c r="T77" s="40"/>
       <c r="U77" s="11" t="s">
         <v>29</v>
       </c>
@@ -5539,7 +5527,7 @@
       <c r="D78" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E78" s="24" t="s">
+      <c r="E78" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F78" s="23" t="s">
@@ -5557,22 +5545,22 @@
       <c r="J78" s="22">
         <v>75</v>
       </c>
-      <c r="K78" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L78" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M78" s="40"/>
+      <c r="K78" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L78" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M78" s="39"/>
       <c r="N78" s="23"/>
       <c r="O78" s="23"/>
-      <c r="P78" s="41"/>
+      <c r="P78" s="40"/>
       <c r="Q78" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R78" s="42"/>
+      <c r="R78" s="41"/>
       <c r="S78" s="23"/>
-      <c r="T78" s="41"/>
+      <c r="T78" s="40"/>
       <c r="U78" s="11" t="s">
         <v>29</v>
       </c>
@@ -5590,7 +5578,7 @@
       <c r="D79" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E79" s="24" t="s">
+      <c r="E79" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F79" s="23" t="s">
@@ -5608,22 +5596,22 @@
       <c r="J79" s="22">
         <v>70</v>
       </c>
-      <c r="K79" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L79" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M79" s="40"/>
+      <c r="K79" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L79" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M79" s="39"/>
       <c r="N79" s="23"/>
       <c r="O79" s="23"/>
-      <c r="P79" s="41"/>
+      <c r="P79" s="40"/>
       <c r="Q79" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R79" s="42"/>
+      <c r="R79" s="41"/>
       <c r="S79" s="23"/>
-      <c r="T79" s="41"/>
+      <c r="T79" s="40"/>
       <c r="U79" s="11" t="s">
         <v>29</v>
       </c>
@@ -5641,7 +5629,7 @@
       <c r="D80" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E80" s="24" t="s">
+      <c r="E80" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F80" s="23" t="s">
@@ -5659,22 +5647,22 @@
       <c r="J80" s="22">
         <v>25</v>
       </c>
-      <c r="K80" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L80" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M80" s="40"/>
+      <c r="K80" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L80" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M80" s="39"/>
       <c r="N80" s="23"/>
       <c r="O80" s="23"/>
-      <c r="P80" s="41"/>
+      <c r="P80" s="40"/>
       <c r="Q80" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R80" s="42"/>
+      <c r="R80" s="41"/>
       <c r="S80" s="23"/>
-      <c r="T80" s="41"/>
+      <c r="T80" s="40"/>
       <c r="U80" s="11" t="s">
         <v>29</v>
       </c>
@@ -5692,7 +5680,7 @@
       <c r="D81" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E81" s="24" t="s">
+      <c r="E81" s="3" t="s">
         <v>143</v>
       </c>
       <c r="F81" s="23" t="s">
@@ -5710,22 +5698,22 @@
       <c r="J81" s="22">
         <v>25</v>
       </c>
-      <c r="K81" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L81" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M81" s="40"/>
+      <c r="K81" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L81" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M81" s="39"/>
       <c r="N81" s="23"/>
       <c r="O81" s="23"/>
-      <c r="P81" s="41"/>
+      <c r="P81" s="40"/>
       <c r="Q81" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R81" s="42"/>
+      <c r="R81" s="41"/>
       <c r="S81" s="23"/>
-      <c r="T81" s="41"/>
+      <c r="T81" s="40"/>
       <c r="U81" s="11" t="s">
         <v>29</v>
       </c>
@@ -5743,7 +5731,7 @@
       <c r="D82" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E82" s="24" t="s">
+      <c r="E82" s="3" t="s">
         <v>161</v>
       </c>
       <c r="F82" s="23" t="s">
@@ -5761,22 +5749,22 @@
       <c r="J82" s="22">
         <v>70</v>
       </c>
-      <c r="K82" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L82" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M82" s="40"/>
+      <c r="K82" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L82" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M82" s="39"/>
       <c r="N82" s="23"/>
       <c r="O82" s="23"/>
-      <c r="P82" s="41"/>
+      <c r="P82" s="40"/>
       <c r="Q82" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R82" s="42"/>
+      <c r="R82" s="41"/>
       <c r="S82" s="23"/>
-      <c r="T82" s="41"/>
+      <c r="T82" s="40"/>
       <c r="U82" s="11" t="s">
         <v>29</v>
       </c>
@@ -5794,7 +5782,7 @@
       <c r="D83" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E83" s="24" t="s">
+      <c r="E83" s="3" t="s">
         <v>161</v>
       </c>
       <c r="F83" s="23" t="s">
@@ -5812,22 +5800,22 @@
       <c r="J83" s="22">
         <v>75</v>
       </c>
-      <c r="K83" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L83" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M83" s="40"/>
+      <c r="K83" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L83" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M83" s="39"/>
       <c r="N83" s="23"/>
       <c r="O83" s="23"/>
-      <c r="P83" s="41"/>
+      <c r="P83" s="40"/>
       <c r="Q83" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R83" s="42"/>
+      <c r="R83" s="41"/>
       <c r="S83" s="23"/>
-      <c r="T83" s="41"/>
+      <c r="T83" s="40"/>
       <c r="U83" s="11" t="s">
         <v>29</v>
       </c>
@@ -5845,7 +5833,7 @@
       <c r="D84" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E84" s="24" t="s">
+      <c r="E84" s="3" t="s">
         <v>161</v>
       </c>
       <c r="F84" s="23" t="s">
@@ -5863,22 +5851,22 @@
       <c r="J84" s="22">
         <v>120</v>
       </c>
-      <c r="K84" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L84" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M84" s="40"/>
+      <c r="K84" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L84" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M84" s="39"/>
       <c r="N84" s="23"/>
       <c r="O84" s="23"/>
-      <c r="P84" s="41"/>
+      <c r="P84" s="40"/>
       <c r="Q84" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R84" s="42"/>
+      <c r="R84" s="41"/>
       <c r="S84" s="23"/>
-      <c r="T84" s="41"/>
+      <c r="T84" s="40"/>
       <c r="U84" s="11" t="s">
         <v>29</v>
       </c>
@@ -5896,7 +5884,7 @@
       <c r="D85" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E85" s="24" t="s">
+      <c r="E85" s="3" t="s">
         <v>161</v>
       </c>
       <c r="F85" s="23" t="s">
@@ -5914,22 +5902,22 @@
       <c r="J85" s="22">
         <v>35</v>
       </c>
-      <c r="K85" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L85" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M85" s="40"/>
+      <c r="K85" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L85" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M85" s="39"/>
       <c r="N85" s="23"/>
       <c r="O85" s="23"/>
-      <c r="P85" s="41"/>
+      <c r="P85" s="40"/>
       <c r="Q85" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R85" s="42"/>
+      <c r="R85" s="41"/>
       <c r="S85" s="23"/>
-      <c r="T85" s="41"/>
+      <c r="T85" s="40"/>
       <c r="U85" s="11" t="s">
         <v>29</v>
       </c>
@@ -5947,7 +5935,7 @@
       <c r="D86" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E86" s="24" t="s">
+      <c r="E86" s="3" t="s">
         <v>161</v>
       </c>
       <c r="F86" s="23" t="s">
@@ -5965,22 +5953,22 @@
       <c r="J86" s="22">
         <v>120</v>
       </c>
-      <c r="K86" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L86" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M86" s="40"/>
+      <c r="K86" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L86" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M86" s="39"/>
       <c r="N86" s="23"/>
       <c r="O86" s="23"/>
-      <c r="P86" s="41"/>
+      <c r="P86" s="40"/>
       <c r="Q86" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R86" s="42"/>
+      <c r="R86" s="41"/>
       <c r="S86" s="23"/>
-      <c r="T86" s="41"/>
+      <c r="T86" s="40"/>
       <c r="U86" s="11" t="s">
         <v>29</v>
       </c>
@@ -5998,7 +5986,7 @@
       <c r="D87" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E87" s="24" t="s">
+      <c r="E87" s="3" t="s">
         <v>170</v>
       </c>
       <c r="F87" s="23" t="s">
@@ -6016,22 +6004,22 @@
       <c r="J87" s="22">
         <v>90</v>
       </c>
-      <c r="K87" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L87" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M87" s="40"/>
+      <c r="K87" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L87" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M87" s="39"/>
       <c r="N87" s="23"/>
       <c r="O87" s="23"/>
-      <c r="P87" s="41"/>
+      <c r="P87" s="40"/>
       <c r="Q87" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R87" s="42"/>
+      <c r="R87" s="41"/>
       <c r="S87" s="23"/>
-      <c r="T87" s="41"/>
+      <c r="T87" s="40"/>
       <c r="U87" s="11" t="s">
         <v>29</v>
       </c>
@@ -6049,7 +6037,7 @@
       <c r="D88" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E88" s="24" t="s">
+      <c r="E88" s="3" t="s">
         <v>170</v>
       </c>
       <c r="F88" s="23" t="s">
@@ -6067,22 +6055,22 @@
       <c r="J88" s="22">
         <v>25</v>
       </c>
-      <c r="K88" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L88" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M88" s="40"/>
+      <c r="K88" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L88" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M88" s="39"/>
       <c r="N88" s="23"/>
       <c r="O88" s="23"/>
-      <c r="P88" s="41"/>
+      <c r="P88" s="40"/>
       <c r="Q88" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R88" s="42"/>
+      <c r="R88" s="41"/>
       <c r="S88" s="23"/>
-      <c r="T88" s="41"/>
+      <c r="T88" s="40"/>
       <c r="U88" s="11" t="s">
         <v>29</v>
       </c>
@@ -6100,7 +6088,7 @@
       <c r="D89" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E89" s="24" t="s">
+      <c r="E89" s="3" t="s">
         <v>170</v>
       </c>
       <c r="F89" s="23" t="s">
@@ -6118,22 +6106,22 @@
       <c r="J89" s="22">
         <v>135</v>
       </c>
-      <c r="K89" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L89" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M89" s="40"/>
+      <c r="K89" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L89" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M89" s="39"/>
       <c r="N89" s="23"/>
       <c r="O89" s="23"/>
-      <c r="P89" s="41"/>
+      <c r="P89" s="40"/>
       <c r="Q89" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R89" s="42"/>
+      <c r="R89" s="41"/>
       <c r="S89" s="23"/>
-      <c r="T89" s="41"/>
+      <c r="T89" s="40"/>
       <c r="U89" s="11" t="s">
         <v>29</v>
       </c>
@@ -6151,7 +6139,7 @@
       <c r="D90" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E90" s="24" t="s">
+      <c r="E90" s="3" t="s">
         <v>170</v>
       </c>
       <c r="F90" s="23" t="s">
@@ -6169,22 +6157,22 @@
       <c r="J90" s="22">
         <v>50</v>
       </c>
-      <c r="K90" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L90" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M90" s="40"/>
+      <c r="K90" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L90" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M90" s="39"/>
       <c r="N90" s="23"/>
       <c r="O90" s="23"/>
-      <c r="P90" s="41"/>
+      <c r="P90" s="40"/>
       <c r="Q90" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R90" s="42"/>
+      <c r="R90" s="41"/>
       <c r="S90" s="23"/>
-      <c r="T90" s="41"/>
+      <c r="T90" s="40"/>
       <c r="U90" s="11" t="s">
         <v>29</v>
       </c>
@@ -6202,7 +6190,7 @@
       <c r="D91" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E91" s="24" t="s">
+      <c r="E91" s="3" t="s">
         <v>170</v>
       </c>
       <c r="F91" s="23" t="s">
@@ -6220,22 +6208,22 @@
       <c r="J91" s="22">
         <v>25</v>
       </c>
-      <c r="K91" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L91" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M91" s="40"/>
+      <c r="K91" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L91" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M91" s="39"/>
       <c r="N91" s="23"/>
       <c r="O91" s="23"/>
-      <c r="P91" s="41"/>
+      <c r="P91" s="40"/>
       <c r="Q91" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R91" s="42"/>
+      <c r="R91" s="41"/>
       <c r="S91" s="23"/>
-      <c r="T91" s="41"/>
+      <c r="T91" s="40"/>
       <c r="U91" s="11" t="s">
         <v>29</v>
       </c>
@@ -6253,7 +6241,7 @@
       <c r="D92" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E92" s="24" t="s">
+      <c r="E92" s="3" t="s">
         <v>170</v>
       </c>
       <c r="F92" s="23" t="s">
@@ -6271,22 +6259,22 @@
       <c r="J92" s="22">
         <v>135</v>
       </c>
-      <c r="K92" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="L92" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="M92" s="40"/>
+      <c r="K92" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L92" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="M92" s="39"/>
       <c r="N92" s="23"/>
       <c r="O92" s="23"/>
-      <c r="P92" s="41"/>
+      <c r="P92" s="40"/>
       <c r="Q92" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R92" s="42"/>
+      <c r="R92" s="41"/>
       <c r="S92" s="23"/>
-      <c r="T92" s="41"/>
+      <c r="T92" s="40"/>
       <c r="U92" s="11" t="s">
         <v>29</v>
       </c>

</xml_diff>